<commit_message>
Daytime QA, clause fills, dedupe, washing calculator
</commit_message>
<xml_diff>
--- a/OBX-Ops/PM Pipeline Tracker [DRAFT].xlsx
+++ b/OBX-Ops/PM Pipeline Tracker [DRAFT].xlsx
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="139">
   <si>
     <t xml:space="preserve">OBX Lot Solutions — PM Call-Sheet &amp; Pipeline Tracker</t>
   </si>
   <si>
-    <t xml:space="preserve">Work top-down. ★ = verified phone, call now. 'verify' = confirm number on website first. Set Status from the dropdown after each call.</t>
+    <t xml:space="preserve">Phones re-verified against official sources May 31, 2026. ★ = verified number, call now. 'verify' = confirm on website (1 left: Crew Cutters). Set Status from the dropdown after each call.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -254,127 +254,154 @@
     <t xml:space="preserve">Referral</t>
   </si>
   <si>
+    <t xml:space="preserve">Resort Realty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM, 615+ homes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corolla→Nags Head + Hatteras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(252) 441-5000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resortrealty.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southern Shores Realty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM, 300+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corolla→Nags Head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(252) 261-2000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">southernshores.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stan White Realty &amp; Const.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM, 300+ (+ construction)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nags Head→Corolla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(252) 441-1515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stanwhiterealty.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maintenance coordinator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM, 300+ (growing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NH,KH,Corolla,KDH,Duck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(866) 316-1843</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keesouterbanks.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maintenance ops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun Realty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM, large</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBX-wide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(252) 441-7035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sunrealtync.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Property-services / maintenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outer Banks Blue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM, 250+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(252) 255-1220</t>
+  </si>
+  <si>
+    <t xml:space="preserve">outerbanksblue.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Village Realty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(252) 480-2224</t>
+  </si>
+  <si>
+    <t xml:space="preserve">villagerealtyobx.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Property-management division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beach Realty &amp; Construction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM (+ construction)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carova→Nags Head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(252) 261-3815</t>
+  </si>
+  <si>
+    <t xml:space="preserve">beachrealtync.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cove Realty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM (smaller/local)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(252) 441-6391</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coverealty.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner / maintenance</t>
+  </si>
+  <si>
     <t xml:space="preserve">verify</t>
   </si>
   <si>
-    <t xml:space="preserve">Resort Realty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRM, 615+ homes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corolla→Nags Head + Hatteras</t>
+    <t xml:space="preserve">Crew Cutters OBX</t>
   </si>
   <si>
     <t xml:space="preserve">verify on site</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resortrealty.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southern Shores Realty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRM, 300+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corolla→Nags Head</t>
-  </si>
-  <si>
-    <t xml:space="preserve">southernshores.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stan White Realty &amp; Const.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRM, 300+ (+ construction)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nags Head→Corolla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stanwhite.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintenance coordinator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KEES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRM, 300+ (growing)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NH,KH,Corolla,KDH,Duck</t>
-  </si>
-  <si>
-    <t xml:space="preserve">keesouterbanks.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintenance ops</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sun Realty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRM, large</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OBX-wide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sunrealtync.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Property-services / maintenance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outer Banks Blue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRM, 250+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">outerbanksblue.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Village Realty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">villagerealtyobx.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Property-management division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beach Realty &amp; Construction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRM (+ construction)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carova→Nags Head</t>
-  </si>
-  <si>
-    <t xml:space="preserve">beachrealtync.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cove Realty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRM (smaller/local)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coverealty.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner / maintenance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crew Cutters OBX</t>
   </si>
   <si>
     <t xml:space="preserve">crewcuttersobx.com</t>
@@ -1449,23 +1476,23 @@
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="G15" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>81</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>49</v>
@@ -1487,20 +1514,20 @@
       <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>76</v>
+      <c r="B16" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C16" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="7" t="s">
         <v>84</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>80</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>85</v>
@@ -1525,8 +1552,8 @@
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>76</v>
+      <c r="B17" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>86</v>
@@ -1538,13 +1565,13 @@
         <v>88</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>38</v>
@@ -1563,26 +1590,26 @@
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>76</v>
+      <c r="B18" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I18" s="4" t="s">
         <v>38</v>
@@ -1601,26 +1628,26 @@
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>76</v>
+      <c r="B19" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>38</v>
@@ -1639,23 +1666,23 @@
       <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>76</v>
+      <c r="B20" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>88</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>49</v>
@@ -1677,26 +1704,26 @@
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>76</v>
+      <c r="B21" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>38</v>
@@ -1715,23 +1742,23 @@
       <c r="A22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>76</v>
+      <c r="B22" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>49</v>
@@ -1753,26 +1780,26 @@
       <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>76</v>
+      <c r="B23" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="I23" s="4" t="s">
         <v>23</v>
@@ -1792,22 +1819,22 @@
         <v>20</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>76</v>
+        <v>123</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>70</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>80</v>
+        <v>125</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>74</v>
@@ -1881,15 +1908,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1910,7 +1937,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Pipeline!K:K,"Contacted")</f>
@@ -1926,7 +1953,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Pipeline!K:K,"Callback")</f>
@@ -1942,7 +1969,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Pipeline!K:K,"Quoted")</f>
@@ -1951,23 +1978,23 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Pipeline!K:K,"Won")</f>
         <v>0</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="E8" s="0" t="n">
         <f aca="false">COUNTIF(Pipeline!B:B,"★")</f>
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">COUNTIF(Pipeline!K:K,"Lost")</f>
@@ -1976,7 +2003,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="B10" s="10" t="n">
         <f aca="false">COUNTA(Pipeline!C5:C24)</f>
@@ -1985,7 +2012,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="B12" s="11" t="n">
         <f aca="false">IFERROR(B9/(B5+B6+B7+B8+B9),0)</f>
@@ -1994,7 +2021,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>